<commit_message>
report: nang so lan do len 10 (Lan1-10) cho bang 5.1/5.2/5.3/5.6 trong file Excel ket qua thuc nghiem
</commit_message>
<xml_diff>
--- a/docs/ket-qua-thuc-nghiem-5.2.xlsx
+++ b/docs/ket-qua-thuc-nghiem-5.2.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="5.1 Quang duong" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="5.2 Xoay goc" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="5.3 Giu huong" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="5.4 Node" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5.5 HC-SR04" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="5.6 Ne vat can" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="5.7 Drift yaw" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.1 Quang duong" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.2 Xoay goc" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.3 Giu huong" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.4 Node" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.5 HC-SR04" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.6 Ne vat can" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.7 Drift yaw" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,31 +477,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. O xanh la = cong thuc tu tinh, dung sua.</t>
+          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. Moi phep do 10 lan (Lan1..Lan10); o xanh la = cong thuc tu tinh, dung sua.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quang lenh (m)</t>
+          <t>Quang duong lenh (m)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -531,15 +536,40 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Lan6</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Lan7</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Lan8</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Lan9</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Lan10</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
           <t>Do thuc TB (m)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Sai so TB (cm)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Sai so (%)</t>
         </is>
@@ -550,30 +580,45 @@
         <v>0.5</v>
       </c>
       <c r="B3" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="3" t="n">
         <v>0.48</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="D3" s="3" t="n">
         <v>0.49</v>
       </c>
-      <c r="D3" s="3" t="n">
-        <v>0.47</v>
-      </c>
       <c r="E3" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="K3" s="3" t="n">
         <v>0.48</v>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="G3" s="4">
-        <f>AVERAGE(B3:F3)</f>
-        <v/>
-      </c>
-      <c r="H3" s="4">
-        <f>ABS(A3-G3)*100</f>
-        <v/>
-      </c>
-      <c r="I3" s="4">
-        <f>ABS(A3-G3)/A3*100</f>
+      <c r="L3" s="4">
+        <f>AVERAGE(B3:K3)</f>
+        <v/>
+      </c>
+      <c r="M3" s="4">
+        <f>ABS(A3-L3)*100</f>
+        <v/>
+      </c>
+      <c r="N3" s="4">
+        <f>ABS(A3-L3)/A3*100</f>
         <v/>
       </c>
     </row>
@@ -582,30 +627,45 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D4" s="3" t="n">
         <v>0.97</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="D4" s="3" t="n">
+      <c r="E4" s="3" t="n">
         <v>0.98</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="F4" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="K4" s="3" t="n">
         <v>0.97</v>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="G4" s="4">
-        <f>AVERAGE(B4:F4)</f>
-        <v/>
-      </c>
-      <c r="H4" s="4">
-        <f>ABS(A4-G4)*100</f>
-        <v/>
-      </c>
-      <c r="I4" s="4">
-        <f>ABS(A4-G4)/A4*100</f>
+      <c r="L4" s="4">
+        <f>AVERAGE(B4:K4)</f>
+        <v/>
+      </c>
+      <c r="M4" s="4">
+        <f>ABS(A4-L4)*100</f>
+        <v/>
+      </c>
+      <c r="N4" s="4">
+        <f>ABS(A4-L4)/A4*100</f>
         <v/>
       </c>
     </row>
@@ -614,10 +674,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1.95</v>
+        <v>1.98</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1.94</v>
+        <v>1.97</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>1.96</v>
@@ -626,24 +686,39 @@
         <v>1.95</v>
       </c>
       <c r="F5" s="3" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="H5" s="3" t="n">
         <v>1.95</v>
       </c>
-      <c r="G5" s="4">
-        <f>AVERAGE(B5:F5)</f>
-        <v/>
-      </c>
-      <c r="H5" s="4">
-        <f>ABS(A5-G5)*100</f>
-        <v/>
-      </c>
-      <c r="I5" s="4">
-        <f>ABS(A5-G5)/A5*100</f>
+      <c r="I5" s="3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="L5" s="4">
+        <f>AVERAGE(B5:K5)</f>
+        <v/>
+      </c>
+      <c r="M5" s="4">
+        <f>ABS(A5-L5)*100</f>
+        <v/>
+      </c>
+      <c r="N5" s="4">
+        <f>ABS(A5-L5)/A5*100</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -655,24 +730,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. O xanh la = cong thuc tu tinh, dung sua.</t>
+          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. Moi phep do 10 lan (Lan1..Lan10); o xanh la = cong thuc tu tinh, dung sua.</t>
         </is>
       </c>
     </row>
@@ -709,15 +789,40 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Lan6</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Lan7</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Lan8</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Lan9</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Lan10</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
           <t>Goc do TB (do)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Sai so TB (do)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Do lech chuan (do)</t>
         </is>
@@ -728,30 +833,45 @@
         <v>45</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>44.5</v>
+        <v>44.7</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>43.8</v>
+        <v>44.6</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>44</v>
+        <v>44.4</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>45</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>43.6</v>
-      </c>
-      <c r="G3" s="4">
-        <f>AVERAGE(B3:F3)</f>
-        <v/>
-      </c>
-      <c r="H3" s="4">
-        <f>ABS(A3-G3)</f>
-        <v/>
-      </c>
-      <c r="I3" s="4">
-        <f>STDEV.S(B3:F3)</f>
+        <v>44.1</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="L3" s="4">
+        <f>AVERAGE(B3:K3)</f>
+        <v/>
+      </c>
+      <c r="M3" s="4">
+        <f>ABS(A3-L3)</f>
+        <v/>
+      </c>
+      <c r="N3" s="4">
+        <f>STDEV.S(B3:K3)</f>
         <v/>
       </c>
     </row>
@@ -760,30 +880,45 @@
         <v>90</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>88.5</v>
+        <v>89</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>89.2</v>
+        <v>87.8</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>87.59999999999999</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>88.90000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="F4" s="3" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>88.09999999999999</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="J4" s="3" t="n">
         <v>88.8</v>
       </c>
-      <c r="G4" s="4">
-        <f>AVERAGE(B4:F4)</f>
-        <v/>
-      </c>
-      <c r="H4" s="4">
-        <f>ABS(A4-G4)</f>
-        <v/>
-      </c>
-      <c r="I4" s="4">
-        <f>STDEV.S(B4:F4)</f>
+      <c r="K4" s="3" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="L4" s="4">
+        <f>AVERAGE(B4:K4)</f>
+        <v/>
+      </c>
+      <c r="M4" s="4">
+        <f>ABS(A4-L4)</f>
+        <v/>
+      </c>
+      <c r="N4" s="4">
+        <f>STDEV.S(B4:K4)</f>
         <v/>
       </c>
     </row>
@@ -792,36 +927,51 @@
         <v>180</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>177.5</v>
+        <v>177.1</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>176</v>
+        <v>176.6</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>178.2</v>
+        <v>176.8</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>175.5</v>
+        <v>178.5</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>177</v>
-      </c>
-      <c r="G5" s="4">
-        <f>AVERAGE(B5:F5)</f>
-        <v/>
-      </c>
-      <c r="H5" s="4">
-        <f>ABS(A5-G5)</f>
-        <v/>
-      </c>
-      <c r="I5" s="4">
-        <f>STDEV.S(B5:F5)</f>
+        <v>177.8</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>177.7</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>178</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>177.1</v>
+      </c>
+      <c r="L5" s="4">
+        <f>AVERAGE(B5:K5)</f>
+        <v/>
+      </c>
+      <c r="M5" s="4">
+        <f>ABS(A5-L5)</f>
+        <v/>
+      </c>
+      <c r="N5" s="4">
+        <f>STDEV.S(B5:K5)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -833,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -844,7 +994,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. O xanh la = cong thuc tu tinh, dung sua.</t>
+          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. Moi phep do 10 lan (Lan1..Lan10); o xanh la = cong thuc tu tinh, dung sua.</t>
         </is>
       </c>
     </row>
@@ -870,7 +1020,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>6</v>
+        <v>8.9</v>
       </c>
       <c r="C3" s="4">
         <f>DEGREES(ATAN(B3/300))</f>
@@ -882,7 +1032,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="C4" s="4">
         <f>DEGREES(ATAN(B4/300))</f>
@@ -894,7 +1044,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>5</v>
+        <v>6.8</v>
       </c>
       <c r="C5" s="4">
         <f>DEGREES(ATAN(B5/300))</f>
@@ -902,17 +1052,101 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="C6" s="4">
+        <f>DEGREES(ATAN(B6/300))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="C7" s="4">
+        <f>DEGREES(ATAN(B7/300))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="C8" s="4">
+        <f>DEGREES(ATAN(B8/300))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="C9" s="4">
+        <f>DEGREES(ATAN(B9/300))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C10" s="4">
+        <f>DEGREES(ATAN(B10/300))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="C11" s="4">
+        <f>DEGREES(ATAN(B11/300))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="C12" s="4">
+        <f>DEGREES(ATAN(B12/300))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Trung binh</t>
         </is>
       </c>
-      <c r="B6" s="4">
-        <f>AVERAGE(B3:B5)</f>
-        <v/>
-      </c>
-      <c r="C6" s="4">
-        <f>AVERAGE(C3:C5)</f>
+      <c r="B13" s="4">
+        <f>AVERAGE(B3:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="4">
+        <f>AVERAGE(C3:C12)</f>
         <v/>
       </c>
     </row>
@@ -943,7 +1177,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. O xanh la = cong thuc tu tinh, dung sua.</t>
+          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. Moi phep do 10 lan (Lan1..Lan10); o xanh la = cong thuc tu tinh, dung sua.</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1292,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. O xanh la = cong thuc tu tinh, dung sua.</t>
+          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. Moi phep do 10 lan (Lan1..Lan10); o xanh la = cong thuc tu tinh, dung sua.</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1187,7 +1421,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. O xanh la = cong thuc tu tinh, dung sua.</t>
+          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. Moi phep do 10 lan (Lan1..Lan10); o xanh la = cong thuc tu tinh, dung sua.</t>
         </is>
       </c>
     </row>
@@ -1218,56 +1452,56 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>28.5</v>
+        <v>26.7</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Co</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
+      <c r="D3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>29.2</v>
+        <v>29.3</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Co</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>27.8</v>
+        <v>29.1</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Co</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
         <v>4</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>26.5</v>
+        <v>27.1</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Khong</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Vat mong (chan ghe), phat hien tre</t>
         </is>
@@ -1278,7 +1512,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>29</v>
+        <v>28.3</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -1288,30 +1522,104 @@
       <c r="D7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Khong</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Vat cham hap thu song, do gan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Ti le thanh cong</t>
         </is>
       </c>
-      <c r="B8" s="4">
-        <f>COUNTIF(C3:C7,"Co")&amp;"/"&amp;COUNTA(C3:C7)&amp;" ("&amp;ROUND(COUNTIF(C3:C7,"Co")/COUNTA(C3:C7)*100,0)&amp;"%)"</f>
-        <v/>
-      </c>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="B13" s="4">
+        <f>COUNTIF(C3:C12,"Co")&amp;"/"&amp;COUNTA(C3:C12)&amp;" ("&amp;ROUND(COUNTIF(C3:C12,"Co")/COUNTA(C3:C12)*100,0)&amp;"%)"</f>
+        <v/>
+      </c>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Kc dung TB (cm)</t>
         </is>
       </c>
-      <c r="B9" s="4">
-        <f>AVERAGE(B3:B7)</f>
-        <v/>
-      </c>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
+      <c r="B14" s="4">
+        <f>AVERAGE(B3:B12)</f>
+        <v/>
+      </c>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1337,7 +1645,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. O xanh la = cong thuc tu tinh, dung sua.</t>
+          <t>SO LIEU MAU - THAY BANG DO THUC TE TRUOC KHI NOP. Moi phep do 10 lan (Lan1..Lan10); o xanh la = cong thuc tu tinh, dung sua.</t>
         </is>
       </c>
     </row>

</xml_diff>